<commit_message>
refactor: padronizar estrutura dos requisitos e atualizar documentação
</commit_message>
<xml_diff>
--- a/public/documents/requirement4/4_4/4_4_modelo_mapa_de_processos.xlsx
+++ b/public/documents/requirement4/4_4/4_4_modelo_mapa_de_processos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiff\integra-sgi\integra-sgi\public\documents\requirement4\4_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52101398-EA68-4972-A466-B8F04D2783D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B35A5F8-5243-4941-821E-F3CE3454B3E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="700" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matriz dos Processos " sheetId="1" r:id="rId1"/>
@@ -1126,6 +1126,15 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1137,15 +1146,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1350,15 +1350,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>83821</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>22861</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>883921</xdr:colOff>
+      <xdr:colOff>800100</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>114301</xdr:rowOff>
+      <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1387,7 +1387,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="83821" y="22861"/>
+          <a:off x="0" y="0"/>
           <a:ext cx="960120" cy="960120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1713,22 +1713,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="57"/>
-      <c r="N2" s="57"/>
-      <c r="O2" s="57"/>
-      <c r="P2" s="57"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="M2" s="60"/>
+      <c r="N2" s="60"/>
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
     </row>
     <row r="3" spans="2:16" ht="10.8" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:16" hidden="1" x14ac:dyDescent="0.3">
@@ -2613,14 +2613,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="61" t="s">
         <v>88</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="E2" s="58" t="s">
+      <c r="C2" s="61"/>
+      <c r="E2" s="61" t="s">
         <v>97</v>
       </c>
-      <c r="F2" s="58"/>
+      <c r="F2" s="61"/>
     </row>
     <row r="4" spans="2:6" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="36" t="s">
@@ -2741,10 +2741,10 @@
       <c r="C12" s="35" t="s">
         <v>78</v>
       </c>
-      <c r="E12" s="59" t="s">
+      <c r="E12" s="62" t="s">
         <v>98</v>
       </c>
-      <c r="F12" s="59"/>
+      <c r="F12" s="62"/>
     </row>
     <row r="13" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B13" s="38" t="s">
@@ -2850,18 +2850,18 @@
   <sheetData>
     <row r="1" spans="2:16" ht="7.2" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:16" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="60" t="s">
+      <c r="B2" s="63" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
-      <c r="K2" s="60"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
     </row>
     <row r="3" spans="2:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L3" s="2" t="s">
@@ -2965,23 +2965,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:17" ht="52.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="58" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
-      <c r="M2" s="62"/>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="58"/>
     </row>
     <row r="4" spans="2:17" ht="17.399999999999999" x14ac:dyDescent="0.25">
       <c r="B4" s="56" t="s">
@@ -3049,19 +3049,19 @@
       <c r="D16" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="F16" s="61" t="s">
+      <c r="F16" s="57" t="s">
         <v>113</v>
       </c>
-      <c r="G16" s="61"/>
-      <c r="H16" s="61"/>
-      <c r="I16" s="61"/>
-      <c r="J16" s="61"/>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="61"/>
-      <c r="N16" s="61"/>
-      <c r="O16" s="61"/>
-      <c r="P16" s="61"/>
+      <c r="G16" s="57"/>
+      <c r="H16" s="57"/>
+      <c r="I16" s="57"/>
+      <c r="J16" s="57"/>
+      <c r="K16" s="57"/>
+      <c r="L16" s="57"/>
+      <c r="M16" s="57"/>
+      <c r="N16" s="57"/>
+      <c r="O16" s="57"/>
+      <c r="P16" s="57"/>
       <c r="Q16" s="34"/>
     </row>
     <row r="17" spans="2:17" ht="55.2" x14ac:dyDescent="0.25">
@@ -3074,19 +3074,19 @@
       <c r="D17" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="F17" s="61" t="s">
+      <c r="F17" s="57" t="s">
         <v>114</v>
       </c>
-      <c r="G17" s="61"/>
-      <c r="H17" s="61"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="61"/>
-      <c r="K17" s="61"/>
-      <c r="L17" s="61"/>
-      <c r="M17" s="61"/>
-      <c r="N17" s="61"/>
-      <c r="O17" s="61"/>
-      <c r="P17" s="61"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="57"/>
+      <c r="I17" s="57"/>
+      <c r="J17" s="57"/>
+      <c r="K17" s="57"/>
+      <c r="L17" s="57"/>
+      <c r="M17" s="57"/>
+      <c r="N17" s="57"/>
+      <c r="O17" s="57"/>
+      <c r="P17" s="57"/>
       <c r="Q17" s="34"/>
     </row>
     <row r="18" spans="2:17" ht="55.2" x14ac:dyDescent="0.25">
@@ -3099,19 +3099,19 @@
       <c r="D18" s="35" t="s">
         <v>107</v>
       </c>
-      <c r="F18" s="61" t="s">
+      <c r="F18" s="57" t="s">
         <v>112</v>
       </c>
-      <c r="G18" s="61"/>
-      <c r="H18" s="61"/>
-      <c r="I18" s="61"/>
-      <c r="J18" s="61"/>
-      <c r="K18" s="61"/>
-      <c r="L18" s="61"/>
-      <c r="M18" s="61"/>
-      <c r="N18" s="61"/>
-      <c r="O18" s="61"/>
-      <c r="P18" s="61"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="57"/>
+      <c r="I18" s="57"/>
+      <c r="J18" s="57"/>
+      <c r="K18" s="57"/>
+      <c r="L18" s="57"/>
+      <c r="M18" s="57"/>
+      <c r="N18" s="57"/>
+      <c r="O18" s="57"/>
+      <c r="P18" s="57"/>
       <c r="Q18" s="34"/>
     </row>
     <row r="19" spans="2:17" ht="41.4" x14ac:dyDescent="0.25">
@@ -3124,19 +3124,19 @@
       <c r="D19" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="F19" s="63" t="s">
+      <c r="F19" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="G19" s="63"/>
-      <c r="H19" s="63"/>
-      <c r="I19" s="63"/>
-      <c r="J19" s="63"/>
-      <c r="K19" s="63"/>
-      <c r="L19" s="63"/>
-      <c r="M19" s="63"/>
-      <c r="N19" s="63"/>
-      <c r="O19" s="63"/>
-      <c r="P19" s="63"/>
+      <c r="G19" s="59"/>
+      <c r="H19" s="59"/>
+      <c r="I19" s="59"/>
+      <c r="J19" s="59"/>
+      <c r="K19" s="59"/>
+      <c r="L19" s="59"/>
+      <c r="M19" s="59"/>
+      <c r="N19" s="59"/>
+      <c r="O19" s="59"/>
+      <c r="P19" s="59"/>
     </row>
     <row r="20" spans="2:17" ht="55.2" x14ac:dyDescent="0.25">
       <c r="B20" s="53" t="s">
@@ -3148,17 +3148,17 @@
       <c r="D20" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F20" s="63"/>
-      <c r="G20" s="63"/>
-      <c r="H20" s="63"/>
-      <c r="I20" s="63"/>
-      <c r="J20" s="63"/>
-      <c r="K20" s="63"/>
-      <c r="L20" s="63"/>
-      <c r="M20" s="63"/>
-      <c r="N20" s="63"/>
-      <c r="O20" s="63"/>
-      <c r="P20" s="63"/>
+      <c r="F20" s="59"/>
+      <c r="G20" s="59"/>
+      <c r="H20" s="59"/>
+      <c r="I20" s="59"/>
+      <c r="J20" s="59"/>
+      <c r="K20" s="59"/>
+      <c r="L20" s="59"/>
+      <c r="M20" s="59"/>
+      <c r="N20" s="59"/>
+      <c r="O20" s="59"/>
+      <c r="P20" s="59"/>
     </row>
     <row r="24" spans="2:17" ht="4.2" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="2:17" ht="6.6" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>